<commit_message>
Add all 18 lessons for the certification discipline
12 lectures with three gates and a 15-question test each, plus six practices built around the Dekanat case: standards and documentation, audit checklist and quality assessment, metrics, testing and security, report, defense. The discipline is now available with all lessons open, and its plan exports to Excel.
</commit_message>
<xml_diff>
--- a/courses/4/is-certification/dist/Учебный_план_Сертификация_информационной_системы.xlsx
+++ b/courses/4/is-certification/dist/Учебный_план_Сертификация_информационной_системы.xlsx
@@ -174,7 +174,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
@@ -195,16 +195,16 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Сертификация ИС»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Сертификация подтверждает соответствие ИС требованиям независимой оценкой. Разбираем участников, виды оценки соответствия, схемы и место сертификации в жизненном цикле системы.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Сертификация ИС</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
+          <t xml:space="preserve">сертификация, оценка соответствия, аккредитация, схема сертификации</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
@@ -225,16 +225,16 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Стандарты и нормативы»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Стандарты задают требования, по которым оценивают ИС. Учимся читать стандарты разных уровней, отличать обязательные нормы от добровольных и находить применимые документы.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Стандарты и нормативы</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t xml:space="preserve">стандарт, технический регламент, ГОСТ Р, ISO/IEC, нормативная ссылка</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">3-4</t>
@@ -255,16 +255,16 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Анализ стандартов; Документация.</t>
+          <t xml:space="preserve">Разбираем стандарт и комплект документации учебной ИС: выделяем применимые требования, строим матрицу соответствия и определяем, каких документов не хватает для оценки.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Анализ стандартов, Документация</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="45" customHeight="1">
+          <t xml:space="preserve">анализ стандарта, матрица соответствия, документация, доказательства</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">5</t>
@@ -285,16 +285,16 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Качество ПО»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Качество это не отсутствие ошибок, а способность продукта удовлетворять заявленные и подразумеваемые потребности. Разбираем обеспечение и контроль качества, проверку и валидацию, цену дефекта.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Качество ПО</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="45" customHeight="1">
+          <t xml:space="preserve">качество, обеспечение качества, контроль качества, верификация, валидация</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">6</t>
@@ -315,16 +315,16 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «ISO/IEC 25010»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Модель качества ISO/IEC 25010 раскладывает качество продукта на восемь характеристик и набор подхарактеристик. Учимся выбирать характеристики под задачу и измерять их.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISO/IEC 25010</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+          <t xml:space="preserve">ISO/IEC 25010, SQuaRE, характеристика качества, подхарактеристика, метрика</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">7-8</t>
@@ -345,16 +345,16 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Чек-лист аудита; Оценка качества.</t>
+          <t xml:space="preserve">Строим чек-лист аудита по ISO/IEC 25010 и оцениваем учебную ИС: собираем свидетельства, выставляем оценки, обосновываем выводы и готовим рекомендации.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Чек-лист аудита, Оценка качества</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
+          <t xml:space="preserve">чек-лист, аудит, оценка качества, свидетельство, рекомендация</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">9</t>
@@ -375,12 +375,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Документация»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Документация это доказательство того, что система сделана и проверена по правилам. Разбираем виды документов, стандарты оформления, управление версиями и прослеживаемость.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Документация</t>
+          <t xml:space="preserve">документация, ГОСТ 19, ГОСТ 34, прослеживаемость, управление версиями</t>
         </is>
       </c>
     </row>
@@ -405,16 +405,16 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практическая работа «Метрики»: выполнение задания, оформление и проверка результата.</t>
+          <t xml:space="preserve">Переводим требования в измеримые показатели: выбираем метрики, задаём способ сбора и пороги, считаем значения для учебной ИС и объясняем результат.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Метрики</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+          <t xml:space="preserve">метрика, порог, измерение, дефектность, доступность</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">11</t>
@@ -435,16 +435,16 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Аудит»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Аудит проверяет систему по свидетельствам, а не по обещаниям. Разбираем программу аудита, роли, выборку, виды находок, отчёт и последующие действия.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аудит</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
+          <t xml:space="preserve">аудит, свидетельство, несоответствие, выборка, корректирующее действие</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">12</t>
@@ -465,16 +465,16 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Оценка соответствия»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Оценка соответствия отвечает на вопрос, выполнены ли требования, и оформляет ответ решением. Проходим этапы сертификации, схемы, испытания, инспекцию и надзор.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Оценка соответствия</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
+          <t xml:space="preserve">оценка соответствия, схема сертификации, испытания, инспекционный контроль, сертификат</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">13-14</t>
@@ -495,16 +495,16 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Совмещённая практическая работа: Тестирование; Безопасность.</t>
+          <t xml:space="preserve">Готовим доказательства для сертификации: план проверок, функциональные и защитные тесты, таблица результатов и вывод о соответствии выбранным требованиям.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тестирование, Безопасность</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="45" customHeight="1">
+          <t xml:space="preserve">тест-план, функциональное тестирование, проверка защиты, свидетельство, вывод</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">15</t>
@@ -525,16 +525,16 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Безопасность»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Безопасность ИС оценивают по защищённости данных и устойчивости к атакам. Разбираем модель угроз, меры ISO/IEC 27001 и 27002, управление уязвимостями и доказательства.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Безопасность</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
+          <t xml:space="preserve">безопасность, модель угроз, ISO/IEC 27001, уязвимость, аудит безопасности</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">16</t>
@@ -555,12 +555,12 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практическая работа «Отчёт»: выполнение задания, оформление и проверка результата.</t>
+          <t xml:space="preserve">Собираем отчёт о сертификации: структура, находки, ссылки на свидетельства, выводы и рекомендации. Учимся писать так, чтобы решение было проверяемым.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отчёт</t>
+          <t xml:space="preserve">отчёт, находка, свидетельство, вывод, рекомендация</t>
         </is>
       </c>
     </row>
@@ -585,16 +585,16 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Тестирование»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Тестирование даёт свидетельства соответствия. Разбираем уровни и виды тестов, тест-планы, протоколы, покрытие и прослеживаемость к требованиям.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Тестирование</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
+          <t xml:space="preserve">тестирование, тест-план, покрытие, прослеживаемость, дефект</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
@@ -615,16 +615,16 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практическая работа «Защита»: выполнение задания, оформление и проверка результата.</t>
+          <t xml:space="preserve">Защищаем результаты оценки: представляем систему, стандарт, свидетельства и вывод, отвечаем на вопросы комиссии и разбираем слабые места собственного кейса.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Защита</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
+          <t xml:space="preserve">защита, презентация, возражение, свидетельство, доработка</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="60" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">19</t>
@@ -645,16 +645,16 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Метрики»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Метрики превращают качество в числа, но только при правильном сборе и интерпретации. Разбираем свойства метрик, базовые значения, пороги и типичные искажения.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Метрики</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="30" customHeight="1">
+          <t xml:space="preserve">метрика, базовое значение, порог, тренд, эффект Гудхарта</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">20</t>
@@ -675,16 +675,16 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Риски»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Риск это событие с вероятностью и последствием. Учимся вести реестр рисков, оценивать их, выбирать обработку и отслеживать остаточный риск в ходе сертификации.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Риски</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="45" customHeight="1">
+          <t xml:space="preserve">риск, вероятность, последствие, реестр рисков, остаточный риск</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="60" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">21</t>
@@ -705,12 +705,12 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Разбор темы «Процедура сертификации»: ключевые понятия, примеры и практические ситуации.</t>
+          <t xml:space="preserve">Собираем процедуру сертификации в единый маршрут: заявка, анализ, испытания, решение, сертификат, надзор и ресертификация. Разбираем типовые причины отказа.</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Процедура сертификации</t>
+          <t xml:space="preserve">процедура, заявка, решение, сертификат, ресертификация</t>
         </is>
       </c>
     </row>

</xml_diff>